<commit_message>
vault backup: 2026-03-27 11:15:23
</commit_message>
<xml_diff>
--- a/附件/精神文明-志愿者活动值班表.xlsx
+++ b/附件/精神文明-志愿者活动值班表.xlsx
@@ -10,7 +10,7 @@
     <sheet name="2023" sheetId="1" r:id="rId1"/>
     <sheet name="2024" sheetId="2" r:id="rId2"/>
     <sheet name="2025" sheetId="3" r:id="rId3"/>
-    <sheet name="2025年社区志愿者活动" sheetId="4" r:id="rId4"/>
+    <sheet name="2026年社区志愿者活动" sheetId="4" r:id="rId4"/>
     <sheet name="Sheet1" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="65">
   <si>
     <t>2023年路段志愿者活动值班表</t>
   </si>
@@ -217,7 +217,10 @@
     <t>重阳节</t>
   </si>
   <si>
-    <t>2025年社区志愿者活动值班表</t>
+    <t>2026年社区志愿者活动值班表</t>
+  </si>
+  <si>
+    <t>2025年</t>
   </si>
   <si>
     <t>2026年</t>
@@ -962,7 +965,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -973,6 +976,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1448,310 +1454,310 @@
   </cols>
   <sheetData>
     <row r="1" ht="27" customHeight="1" spans="1:17">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
-      <c r="K1" s="28">
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="28"/>
+      <c r="K1" s="29">
         <v>2024</v>
       </c>
-      <c r="L1" s="28"/>
-      <c r="M1" s="28"/>
-      <c r="N1" s="28"/>
-      <c r="O1" s="28"/>
-      <c r="P1" s="28"/>
-      <c r="Q1" s="28"/>
+      <c r="L1" s="29"/>
+      <c r="M1" s="29"/>
+      <c r="N1" s="29"/>
+      <c r="O1" s="29"/>
+      <c r="P1" s="29"/>
+      <c r="Q1" s="29"/>
     </row>
     <row r="2" ht="19" customHeight="1" spans="1:17">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" ht="19" customHeight="1" spans="1:17">
-      <c r="A3" s="5">
+      <c r="A3" s="6">
         <v>1</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="11"/>
-      <c r="D3" s="8">
+      <c r="C3" s="12"/>
+      <c r="D3" s="9">
         <v>44967</v>
       </c>
-      <c r="E3" s="8">
+      <c r="E3" s="9">
         <v>45072</v>
       </c>
-      <c r="F3" s="8">
+      <c r="F3" s="9">
         <v>45170</v>
       </c>
-      <c r="G3" s="8">
+      <c r="G3" s="9">
         <v>45247</v>
       </c>
     </row>
     <row r="4" ht="19" customHeight="1" spans="1:17">
-      <c r="A4" s="5">
+      <c r="A4" s="6">
         <v>2</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="11"/>
-      <c r="D4" s="8">
+      <c r="C4" s="12"/>
+      <c r="D4" s="9">
         <v>44994</v>
       </c>
-      <c r="E4" s="8">
+      <c r="E4" s="9">
         <v>45086</v>
       </c>
-      <c r="F4" s="8">
+      <c r="F4" s="9">
         <v>45177</v>
       </c>
     </row>
     <row r="5" ht="19" customHeight="1" spans="1:17">
-      <c r="A5" s="5">
+      <c r="A5" s="6">
         <v>3</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="7"/>
-      <c r="D5" s="24"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="25"/>
     </row>
     <row r="6" ht="19" customHeight="1" spans="1:17">
-      <c r="A6" s="5"/>
-      <c r="B6" s="10" t="s">
+      <c r="A6" s="6"/>
+      <c r="B6" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="9"/>
-      <c r="D6" s="24"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="25"/>
     </row>
     <row r="7" ht="19" customHeight="1" spans="1:17">
-      <c r="A7" s="5">
+      <c r="A7" s="6">
         <v>4</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="11"/>
-      <c r="D7" s="8">
+      <c r="C7" s="12"/>
+      <c r="D7" s="9">
         <v>45008</v>
       </c>
-      <c r="E7" s="8">
+      <c r="E7" s="9">
         <v>45093</v>
       </c>
-      <c r="F7" s="8">
+      <c r="F7" s="9">
         <v>45184</v>
       </c>
-      <c r="G7" s="8">
+      <c r="G7" s="9">
         <v>45261</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="1:17">
-      <c r="A8" s="5">
+      <c r="A8" s="6">
         <v>5</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="11"/>
-      <c r="D8" s="8">
+      <c r="C8" s="12"/>
+      <c r="D8" s="9">
         <v>44987</v>
       </c>
-      <c r="E8" s="8">
+      <c r="E8" s="9">
         <v>45120</v>
       </c>
-      <c r="F8" s="8">
+      <c r="F8" s="9">
         <v>45188</v>
       </c>
-      <c r="G8" s="8">
+      <c r="G8" s="9">
         <v>45254</v>
       </c>
-      <c r="K8" s="24"/>
+      <c r="K8" s="25"/>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:17">
-      <c r="A9" s="5">
+      <c r="A9" s="6">
         <v>6</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="11"/>
-      <c r="D9" s="8">
+      <c r="C9" s="12"/>
+      <c r="D9" s="9">
         <v>44988</v>
       </c>
-      <c r="E9" s="8">
+      <c r="E9" s="9">
         <v>45107</v>
       </c>
-      <c r="F9" s="8">
+      <c r="F9" s="9">
         <v>45187</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:17">
-      <c r="A10" s="5">
+      <c r="A10" s="6">
         <v>7</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="11"/>
-      <c r="D10" s="8">
+      <c r="C10" s="12"/>
+      <c r="D10" s="9">
         <v>45016</v>
       </c>
-      <c r="E10" s="8">
+      <c r="E10" s="9">
         <v>45128</v>
       </c>
-      <c r="F10" s="8">
+      <c r="F10" s="9">
         <v>45189</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:17">
-      <c r="A11" s="5">
+      <c r="A11" s="6">
         <v>8</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="11"/>
-      <c r="D11" s="8">
+      <c r="C11" s="12"/>
+      <c r="D11" s="9">
         <v>45022</v>
       </c>
-      <c r="E11" s="8">
+      <c r="E11" s="9">
         <v>45162</v>
       </c>
-      <c r="F11" s="8">
+      <c r="F11" s="9">
         <v>45190</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:17">
-      <c r="A12" s="5"/>
-      <c r="B12" s="21" t="s">
+      <c r="A12" s="6"/>
+      <c r="B12" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="C12" s="11"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8">
+      <c r="C12" s="12"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9">
         <v>45163</v>
       </c>
-      <c r="F12" s="8">
+      <c r="F12" s="9">
         <v>45191</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:17">
-      <c r="A13" s="5">
+      <c r="A13" s="6">
         <v>9</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="11"/>
-      <c r="D13" s="8">
+      <c r="C13" s="12"/>
+      <c r="D13" s="9">
         <v>44987</v>
       </c>
-      <c r="E13" s="8">
+      <c r="E13" s="9">
         <v>45135</v>
       </c>
-      <c r="F13" s="8">
+      <c r="F13" s="9">
         <v>45212</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:17">
-      <c r="A14" s="25">
+      <c r="A14" s="26">
         <v>10</v>
       </c>
-      <c r="B14" s="18" t="s">
+      <c r="B14" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="19"/>
-      <c r="D14" s="29">
+      <c r="C14" s="20"/>
+      <c r="D14" s="30">
         <v>45030</v>
       </c>
-      <c r="E14" s="29">
+      <c r="E14" s="30">
         <v>45142</v>
       </c>
-      <c r="F14" s="30" t="s">
+      <c r="F14" s="31" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:17">
-      <c r="A15" s="25">
+      <c r="A15" s="26">
         <v>11</v>
       </c>
-      <c r="B15" s="18" t="s">
+      <c r="B15" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="C15" s="19"/>
-      <c r="D15" s="29">
+      <c r="C15" s="20"/>
+      <c r="D15" s="30">
         <v>45037</v>
       </c>
-      <c r="E15" s="29">
+      <c r="E15" s="30">
         <v>45149</v>
       </c>
-      <c r="F15" s="31"/>
+      <c r="F15" s="32"/>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:17">
-      <c r="A16" s="5">
+      <c r="A16" s="6">
         <v>12</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="C16" s="11"/>
-      <c r="D16" s="8">
+      <c r="C16" s="12"/>
+      <c r="D16" s="9">
         <v>45044</v>
       </c>
-      <c r="E16" s="32">
+      <c r="E16" s="33">
         <v>45156</v>
       </c>
-      <c r="F16" s="8">
+      <c r="F16" s="9">
         <v>45226</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:9">
-      <c r="A17" s="5">
+      <c r="A17" s="6">
         <v>13</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="C17" s="11"/>
-      <c r="D17" s="8">
+      <c r="C17" s="12"/>
+      <c r="D17" s="9">
         <v>45058</v>
       </c>
-      <c r="E17" s="32">
+      <c r="E17" s="33">
         <v>45183</v>
       </c>
-      <c r="F17" s="8">
+      <c r="F17" s="9">
         <v>45233</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:9">
-      <c r="A18" s="5">
+      <c r="A18" s="6">
         <v>14</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="B18" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="C18" s="11"/>
-      <c r="D18" s="8">
+      <c r="C18" s="12"/>
+      <c r="D18" s="9">
         <v>45065</v>
       </c>
-      <c r="E18" s="8">
+      <c r="E18" s="9">
         <v>45219</v>
       </c>
-      <c r="F18" s="8">
+      <c r="F18" s="9">
         <v>45240</v>
       </c>
     </row>
@@ -1763,147 +1769,147 @@
       <c r="C22" s="3"/>
     </row>
     <row r="23" ht="19" customHeight="1" spans="1:9">
-      <c r="A23" s="4" t="s">
+      <c r="A23" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C23" s="5" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="24" ht="19" customHeight="1" spans="1:9">
-      <c r="A24" s="5">
+      <c r="A24" s="6">
         <v>1</v>
       </c>
-      <c r="B24" s="10" t="s">
+      <c r="B24" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="C24" s="11"/>
-      <c r="D24" s="8">
+      <c r="C24" s="12"/>
+      <c r="D24" s="9">
         <v>44967</v>
       </c>
-      <c r="E24" s="8">
+      <c r="E24" s="9">
         <v>45016</v>
       </c>
-      <c r="F24" s="8">
+      <c r="F24" s="9">
         <v>45058</v>
       </c>
       <c r="G24" t="s">
         <v>23</v>
       </c>
-      <c r="H24" s="8">
+      <c r="H24" s="9">
         <v>45163</v>
       </c>
-      <c r="I24" s="8">
+      <c r="I24" s="9">
         <v>45222</v>
       </c>
     </row>
     <row r="25" ht="19" customHeight="1" spans="1:9">
-      <c r="A25" s="5">
+      <c r="A25" s="6">
         <v>2</v>
       </c>
-      <c r="B25" s="10" t="s">
+      <c r="B25" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="C25" s="11"/>
-      <c r="D25" s="8">
+      <c r="C25" s="12"/>
+      <c r="D25" s="9">
         <v>44988</v>
       </c>
-      <c r="E25" s="8">
+      <c r="E25" s="9">
         <v>45022</v>
       </c>
-      <c r="F25" s="8">
+      <c r="F25" s="9">
         <v>45072</v>
       </c>
-      <c r="G25" s="33">
+      <c r="G25" s="34">
         <v>45142</v>
       </c>
-      <c r="H25" s="8">
+      <c r="H25" s="9">
         <v>45212</v>
       </c>
     </row>
     <row r="26" ht="19" customHeight="1" spans="1:9">
-      <c r="A26" s="5">
+      <c r="A26" s="6">
         <v>3</v>
       </c>
-      <c r="B26" s="10" t="s">
+      <c r="B26" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="C26" s="7"/>
-      <c r="D26" s="26">
+      <c r="C26" s="8"/>
+      <c r="D26" s="27">
         <v>44994</v>
       </c>
-      <c r="E26" s="26">
+      <c r="E26" s="27">
         <v>45030</v>
       </c>
-      <c r="F26" s="26">
+      <c r="F26" s="27">
         <v>45107</v>
       </c>
-      <c r="G26" s="26">
+      <c r="G26" s="27">
         <v>45156</v>
       </c>
-      <c r="H26" s="26">
+      <c r="H26" s="27">
         <v>45184</v>
       </c>
-      <c r="I26" s="26">
+      <c r="I26" s="27">
         <v>45247</v>
       </c>
     </row>
     <row r="27" ht="19" customHeight="1" spans="1:9">
-      <c r="A27" s="5"/>
-      <c r="B27" s="10" t="s">
+      <c r="A27" s="6"/>
+      <c r="B27" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="C27" s="9"/>
-      <c r="D27" s="24"/>
-      <c r="E27" s="24"/>
-      <c r="F27" s="24"/>
-      <c r="G27" s="24"/>
-      <c r="H27" s="24"/>
-      <c r="I27" s="24"/>
+      <c r="C27" s="10"/>
+      <c r="D27" s="25"/>
+      <c r="E27" s="25"/>
+      <c r="F27" s="25"/>
+      <c r="G27" s="25"/>
+      <c r="H27" s="25"/>
+      <c r="I27" s="25"/>
     </row>
     <row r="28" ht="19" customHeight="1" spans="1:9">
-      <c r="A28" s="34">
+      <c r="A28" s="35">
         <v>4</v>
       </c>
-      <c r="B28" s="35" t="s">
+      <c r="B28" s="36" t="s">
         <v>27</v>
       </c>
-      <c r="C28" s="36"/>
-      <c r="D28" s="37">
+      <c r="C28" s="37"/>
+      <c r="D28" s="38">
         <v>44994</v>
       </c>
-      <c r="E28" s="37">
+      <c r="E28" s="38">
         <v>45037</v>
       </c>
-      <c r="F28" s="37">
+      <c r="F28" s="38">
         <v>45120</v>
       </c>
-      <c r="G28" s="37">
+      <c r="G28" s="38">
         <v>45183</v>
       </c>
-      <c r="H28" s="8"/>
+      <c r="H28" s="9"/>
     </row>
     <row r="29" ht="19" customHeight="1" spans="1:9">
-      <c r="A29" s="5">
+      <c r="A29" s="6">
         <v>5</v>
       </c>
-      <c r="B29" s="10" t="s">
+      <c r="B29" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="C29" s="11"/>
-      <c r="D29" s="8">
+      <c r="C29" s="12"/>
+      <c r="D29" s="9">
         <v>45008</v>
       </c>
-      <c r="E29" s="8">
+      <c r="E29" s="9">
         <v>45065</v>
       </c>
-      <c r="F29" s="8">
+      <c r="F29" s="9">
         <v>45149</v>
       </c>
-      <c r="G29" s="8">
+      <c r="G29" s="9">
         <v>45219</v>
       </c>
     </row>
@@ -1953,11 +1959,11 @@
   </cols>
   <sheetData>
     <row r="1" ht="17.4" spans="1:11">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
       <c r="D1" t="s">
         <v>30</v>
       </c>
@@ -1969,31 +1975,31 @@
       </c>
     </row>
     <row r="2" spans="1:11">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:11">
-      <c r="A3" s="5">
+      <c r="A3" s="6">
         <v>1</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="11"/>
-      <c r="D3" s="8">
+      <c r="C3" s="12"/>
+      <c r="D3" s="9">
         <v>45247</v>
       </c>
-      <c r="F3" s="8">
+      <c r="F3" s="9">
         <v>45485</v>
       </c>
-      <c r="G3" s="8">
+      <c r="G3" s="9">
         <v>45590</v>
       </c>
       <c r="H3" t="s">
@@ -2001,308 +2007,308 @@
       </c>
     </row>
     <row r="4" spans="1:11">
-      <c r="A4" s="5">
+      <c r="A4" s="6">
         <v>2</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="11"/>
-      <c r="E4" s="8">
+      <c r="C4" s="12"/>
+      <c r="E4" s="9">
         <v>45303</v>
       </c>
-      <c r="F4" s="8">
+      <c r="F4" s="9">
         <v>45471</v>
       </c>
-      <c r="G4" s="8">
+      <c r="G4" s="9">
         <v>45596</v>
       </c>
-      <c r="H4" s="8">
+      <c r="H4" s="9">
         <v>45709</v>
       </c>
     </row>
     <row r="5" spans="1:11">
-      <c r="A5" s="5">
+      <c r="A5" s="6">
         <v>3</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="7"/>
-      <c r="F5" s="24"/>
+      <c r="C5" s="8"/>
+      <c r="F5" s="25"/>
       <c r="G5" t="s">
         <v>34</v>
       </c>
-      <c r="H5" s="8">
+      <c r="H5" s="9">
         <v>45716</v>
       </c>
     </row>
     <row r="6" ht="28.8" spans="1:11">
-      <c r="A6" s="5"/>
-      <c r="B6" s="10" t="s">
+      <c r="A6" s="6"/>
+      <c r="B6" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="9"/>
-      <c r="F6" s="24"/>
-      <c r="G6" s="22" t="s">
+      <c r="C6" s="10"/>
+      <c r="F6" s="25"/>
+      <c r="G6" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="H6" s="8">
+      <c r="H6" s="9">
         <v>45716</v>
       </c>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="5">
+      <c r="A7" s="6">
         <v>4</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="11"/>
-      <c r="D7" s="8">
+      <c r="C7" s="12"/>
+      <c r="D7" s="9">
         <v>45261</v>
       </c>
-      <c r="F7" s="8">
+      <c r="F7" s="9">
         <v>45499</v>
       </c>
-      <c r="G7" s="8">
+      <c r="G7" s="9">
         <v>45604</v>
       </c>
-      <c r="H7" s="8">
+      <c r="H7" s="9">
         <v>45723</v>
       </c>
     </row>
     <row r="8" spans="1:11">
-      <c r="A8" s="5">
+      <c r="A8" s="6">
         <v>5</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="11"/>
-      <c r="D8" s="8">
+      <c r="C8" s="12"/>
+      <c r="D8" s="9">
         <v>45254</v>
       </c>
-      <c r="F8" s="8">
+      <c r="F8" s="9">
         <v>45506</v>
       </c>
-      <c r="G8" s="8">
+      <c r="G8" s="9">
         <v>45618</v>
       </c>
     </row>
     <row r="9" spans="1:11">
-      <c r="A9" s="5">
+      <c r="A9" s="6">
         <v>6</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="11"/>
-      <c r="E9" s="8">
+      <c r="C9" s="12"/>
+      <c r="E9" s="9">
         <v>45352</v>
       </c>
-      <c r="F9" s="8">
+      <c r="F9" s="9">
         <v>45513</v>
       </c>
-      <c r="G9" s="8">
+      <c r="G9" s="9">
         <v>45610</v>
       </c>
-      <c r="H9" s="8">
+      <c r="H9" s="9">
         <v>45736</v>
       </c>
     </row>
     <row r="10" ht="15.6" spans="1:11">
-      <c r="A10" s="5"/>
-      <c r="B10" s="10" t="s">
+      <c r="A10" s="6"/>
+      <c r="B10" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8">
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9">
         <v>45624</v>
       </c>
-      <c r="I10" s="13" t="s">
+      <c r="I10" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="J10" s="14" t="s">
+      <c r="J10" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="K10" s="8">
+      <c r="K10" s="9">
         <v>45624</v>
       </c>
     </row>
     <row r="11" ht="15.6" spans="1:11">
-      <c r="A11" s="5">
+      <c r="A11" s="6">
         <v>7</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="C11" s="11"/>
-      <c r="E11" s="8">
+      <c r="C11" s="12"/>
+      <c r="E11" s="9">
         <v>45359</v>
       </c>
-      <c r="F11" s="8">
+      <c r="F11" s="9">
         <v>45519</v>
       </c>
-      <c r="G11" s="8">
+      <c r="G11" s="9">
         <v>45632</v>
       </c>
-      <c r="I11" s="13" t="s">
+      <c r="I11" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="J11" s="14" t="s">
+      <c r="J11" s="15" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="12" ht="15.6" spans="1:11">
-      <c r="A12" s="5">
+      <c r="A12" s="6">
         <v>8</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="C12" s="11"/>
-      <c r="E12" s="8">
+      <c r="C12" s="12"/>
+      <c r="E12" s="9">
         <v>45373</v>
       </c>
-      <c r="F12" s="8">
+      <c r="F12" s="9">
         <v>45527</v>
       </c>
-      <c r="G12" s="8">
+      <c r="G12" s="9">
         <v>45638</v>
       </c>
-      <c r="I12" s="13" t="s">
+      <c r="I12" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="J12" s="14" t="s">
+      <c r="J12" s="15" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="5"/>
-      <c r="B13" s="21" t="s">
+      <c r="A13" s="6"/>
+      <c r="B13" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="11"/>
-      <c r="E13" s="8">
+      <c r="C13" s="12"/>
+      <c r="E13" s="9">
         <v>45401</v>
       </c>
       <c r="F13" t="s">
         <v>45</v>
       </c>
-      <c r="G13" s="8">
+      <c r="G13" s="9">
         <v>45645</v>
       </c>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="5">
+      <c r="A14" s="6">
         <v>9</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="C14" s="11"/>
-      <c r="E14" s="8">
+      <c r="C14" s="12"/>
+      <c r="E14" s="9">
         <v>45408</v>
       </c>
-      <c r="F14" s="8">
+      <c r="F14" s="9">
         <v>45541</v>
       </c>
-      <c r="G14" s="8">
+      <c r="G14" s="9">
         <v>45653</v>
       </c>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="25">
+      <c r="A15" s="26">
         <v>10</v>
       </c>
-      <c r="B15" s="18" t="s">
+      <c r="B15" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="C15" s="19"/>
-      <c r="E15" s="8">
+      <c r="C15" s="20"/>
+      <c r="E15" s="9">
         <v>45423</v>
       </c>
       <c r="F15" t="s">
         <v>46</v>
       </c>
-      <c r="G15" s="8">
+      <c r="G15" s="9">
         <v>45660</v>
       </c>
     </row>
     <row r="16" spans="1:11">
-      <c r="A16" s="25">
+      <c r="A16" s="26">
         <v>11</v>
       </c>
-      <c r="B16" s="18" t="s">
+      <c r="B16" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="C16" s="19"/>
-      <c r="E16" s="8">
+      <c r="C16" s="20"/>
+      <c r="E16" s="9">
         <v>45429</v>
       </c>
       <c r="F16" t="s">
         <v>47</v>
       </c>
-      <c r="G16" s="8">
+      <c r="G16" s="9">
         <v>45667</v>
       </c>
     </row>
     <row r="17" spans="1:14">
-      <c r="A17" s="25">
+      <c r="A17" s="26">
         <v>12</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="C17" s="19"/>
-      <c r="E17" s="8">
+      <c r="C17" s="20"/>
+      <c r="E17" s="9">
         <v>45443</v>
       </c>
-      <c r="F17" s="8">
+      <c r="F17" s="9">
         <v>45562</v>
       </c>
-      <c r="G17" s="8">
+      <c r="G17" s="9">
         <v>45674</v>
       </c>
     </row>
     <row r="18" spans="1:14">
-      <c r="A18" s="25">
+      <c r="A18" s="26">
         <v>13</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="B18" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="C18" s="11"/>
-      <c r="E18" s="8">
+      <c r="C18" s="12"/>
+      <c r="E18" s="9">
         <v>45450</v>
       </c>
-      <c r="F18" s="8">
+      <c r="F18" s="9">
         <v>45576</v>
       </c>
-      <c r="G18" s="8">
+      <c r="G18" s="9">
         <v>45681</v>
       </c>
     </row>
     <row r="19" spans="1:14">
-      <c r="A19" s="5">
+      <c r="A19" s="6">
         <v>14</v>
       </c>
-      <c r="B19" s="10" t="s">
+      <c r="B19" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="C19" s="11"/>
-      <c r="E19" s="8">
+      <c r="C19" s="12"/>
+      <c r="E19" s="9">
         <v>45464</v>
       </c>
-      <c r="F19" s="8">
+      <c r="F19" s="9">
         <v>45582</v>
       </c>
-      <c r="G19" s="8">
+      <c r="G19" s="9">
         <v>45730</v>
       </c>
     </row>
@@ -2320,197 +2326,197 @@
       </c>
     </row>
     <row r="24" spans="1:14">
-      <c r="A24" s="4" t="s">
+      <c r="A24" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="C24" s="5" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="25" spans="1:14">
-      <c r="A25" s="5">
+      <c r="A25" s="6">
         <v>1</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="C25" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="D25" s="8">
+      <c r="D25" s="9">
         <v>45222</v>
       </c>
-      <c r="F25" s="8">
+      <c r="F25" s="9">
         <v>45408</v>
       </c>
-      <c r="G25" s="8">
+      <c r="G25" s="9">
         <v>45450</v>
       </c>
-      <c r="H25" s="8">
+      <c r="H25" s="9">
         <v>45527</v>
       </c>
       <c r="I25" t="s">
         <v>50</v>
       </c>
-      <c r="J25" s="8">
+      <c r="J25" s="9">
         <v>45596</v>
       </c>
-      <c r="K25" s="8">
+      <c r="K25" s="9">
         <v>45624</v>
       </c>
-      <c r="L25" s="8">
+      <c r="L25" s="9">
         <v>45653</v>
       </c>
-      <c r="M25" s="8">
+      <c r="M25" s="9">
         <v>45681</v>
       </c>
-      <c r="N25" s="8">
+      <c r="N25" s="9">
         <v>45723</v>
       </c>
     </row>
     <row r="26" spans="1:14">
-      <c r="A26" s="5">
+      <c r="A26" s="6">
         <v>3</v>
       </c>
-      <c r="B26" s="6" t="s">
+      <c r="B26" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C26" s="7" t="s">
+      <c r="C26" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="D26" s="26">
+      <c r="D26" s="27">
         <v>45247</v>
       </c>
-      <c r="F26" s="26">
+      <c r="F26" s="27">
         <v>45443</v>
       </c>
-      <c r="H26" s="8">
+      <c r="H26" s="9">
         <v>45541</v>
       </c>
-      <c r="I26" s="8">
+      <c r="I26" s="9">
         <v>45582</v>
       </c>
-      <c r="J26" s="8">
+      <c r="J26" s="9">
         <v>45604</v>
       </c>
-      <c r="K26" s="8">
+      <c r="K26" s="9">
         <v>45632</v>
       </c>
-      <c r="L26" s="8">
+      <c r="L26" s="9">
         <v>45660</v>
       </c>
-      <c r="M26" s="8">
+      <c r="M26" s="9">
         <v>45701</v>
       </c>
-      <c r="N26" s="8">
+      <c r="N26" s="9">
         <v>45730</v>
       </c>
     </row>
     <row r="27" spans="1:14">
-      <c r="A27" s="5">
+      <c r="A27" s="6">
         <v>4</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C27" s="9"/>
-      <c r="D27" s="24"/>
-      <c r="F27" s="24"/>
-      <c r="H27" s="8">
+      <c r="C27" s="10"/>
+      <c r="D27" s="25"/>
+      <c r="F27" s="25"/>
+      <c r="H27" s="9">
         <v>45541</v>
       </c>
-      <c r="I27" s="8">
+      <c r="I27" s="9">
         <v>45582</v>
       </c>
-      <c r="J27" s="8">
+      <c r="J27" s="9">
         <v>45604</v>
       </c>
-      <c r="K27" s="8">
+      <c r="K27" s="9">
         <v>45632</v>
       </c>
-      <c r="L27" s="8">
+      <c r="L27" s="9">
         <v>45660</v>
       </c>
-      <c r="M27" s="8">
+      <c r="M27" s="9">
         <v>45701</v>
       </c>
-      <c r="N27" s="8">
+      <c r="N27" s="9">
         <v>45730</v>
       </c>
     </row>
     <row r="28" spans="1:14">
-      <c r="A28" s="5">
+      <c r="A28" s="6">
         <v>2</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="B28" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="C28" s="5" t="s">
+      <c r="C28" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="E28" s="8">
+      <c r="E28" s="9">
         <v>45358</v>
       </c>
-      <c r="F28" s="8">
+      <c r="F28" s="9">
         <v>45423</v>
       </c>
       <c r="H28" t="s">
         <v>52</v>
       </c>
-      <c r="I28" s="8" t="s">
+      <c r="I28" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="J28" s="8">
+      <c r="J28" s="9">
         <v>45610</v>
       </c>
-      <c r="K28" s="8">
+      <c r="K28" s="9">
         <v>45638</v>
       </c>
-      <c r="L28" s="8">
+      <c r="L28" s="9">
         <v>45667</v>
       </c>
-      <c r="M28" s="8">
+      <c r="M28" s="9">
         <v>45709</v>
       </c>
-      <c r="N28" s="8">
+      <c r="N28" s="9">
         <v>45736</v>
       </c>
     </row>
     <row r="29" spans="1:14">
-      <c r="A29" s="5">
+      <c r="A29" s="6">
         <v>5</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C29" s="5" t="s">
+      <c r="C29" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="E29" s="8">
+      <c r="E29" s="9">
         <v>45401</v>
       </c>
-      <c r="F29" s="8">
+      <c r="F29" s="9">
         <v>45464</v>
       </c>
       <c r="H29" t="s">
         <v>55</v>
       </c>
-      <c r="I29" s="8">
+      <c r="I29" s="9">
         <v>45590</v>
       </c>
-      <c r="J29" s="8">
+      <c r="J29" s="9">
         <v>45618</v>
       </c>
-      <c r="K29" s="8">
+      <c r="K29" s="9">
         <v>45645</v>
       </c>
-      <c r="L29" s="8">
+      <c r="L29" s="9">
         <v>45674</v>
       </c>
-      <c r="M29" s="8">
+      <c r="M29" s="9">
         <v>45716</v>
       </c>
     </row>
@@ -2556,66 +2562,66 @@
       <c r="C39" s="3"/>
     </row>
     <row r="40" spans="1:8">
-      <c r="A40" s="4" t="s">
+      <c r="A40" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B40" s="4" t="s">
+      <c r="B40" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C40" s="4" t="s">
+      <c r="C40" s="5" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="41" spans="1:8">
-      <c r="A41" s="5">
+      <c r="A41" s="6">
         <v>1</v>
       </c>
-      <c r="B41" s="6" t="s">
+      <c r="B41" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C41" s="5" t="s">
+      <c r="C41" s="6" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="42" spans="1:8">
-      <c r="A42" s="5">
+      <c r="A42" s="6">
         <v>3</v>
       </c>
-      <c r="B42" s="6" t="s">
+      <c r="B42" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C42" s="7" t="s">
+      <c r="C42" s="8" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="43" spans="1:8">
-      <c r="A43" s="5">
+      <c r="A43" s="6">
         <v>4</v>
       </c>
-      <c r="B43" s="6" t="s">
+      <c r="B43" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C43" s="9"/>
+      <c r="C43" s="10"/>
     </row>
     <row r="44" spans="1:8">
-      <c r="A44" s="5">
+      <c r="A44" s="6">
         <v>2</v>
       </c>
-      <c r="B44" s="6" t="s">
+      <c r="B44" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="C44" s="5" t="s">
+      <c r="C44" s="6" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="45" spans="1:8">
-      <c r="A45" s="5">
+      <c r="A45" s="6">
         <v>5</v>
       </c>
-      <c r="B45" s="6" t="s">
+      <c r="B45" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C45" s="5" t="s">
+      <c r="C45" s="6" t="s">
         <v>54</v>
       </c>
     </row>
@@ -2658,11 +2664,11 @@
   </cols>
   <sheetData>
     <row r="1" ht="17.4" spans="1:16">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
       <c r="D1" t="s">
         <v>30</v>
       </c>
@@ -2671,242 +2677,242 @@
       </c>
     </row>
     <row r="2" ht="15.6" spans="1:16">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="J2" s="10" t="s">
+      <c r="J2" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="K2" s="11" t="s">
+      <c r="K2" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="L2" s="8">
+      <c r="L2" s="9">
         <v>45743</v>
       </c>
-      <c r="M2" s="8"/>
-      <c r="O2" s="13" t="s">
+      <c r="M2" s="9"/>
+      <c r="O2" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="P2" s="14" t="s">
+      <c r="P2" s="15" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="3" ht="15.6" spans="1:16">
-      <c r="A3" s="5">
+      <c r="A3" s="6">
         <v>1</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="11"/>
-      <c r="D3" s="8"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="9"/>
       <c r="E3" t="s">
         <v>33</v>
       </c>
-      <c r="F3" s="8"/>
-      <c r="O3" s="13" t="s">
+      <c r="F3" s="9"/>
+      <c r="O3" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="P3" s="14" t="s">
+      <c r="P3" s="15" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="4" ht="15.6" spans="1:16">
-      <c r="A4" s="5">
+      <c r="A4" s="6">
         <v>2</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="11"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="8">
+      <c r="C4" s="12"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9">
         <v>45709</v>
       </c>
-      <c r="F4" s="8"/>
-      <c r="O4" s="13" t="s">
+      <c r="F4" s="9"/>
+      <c r="O4" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="P4" s="14" t="s">
+      <c r="P4" s="15" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:16">
-      <c r="A5" s="5">
+      <c r="A5" s="6">
         <v>3</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="7"/>
-      <c r="E5" s="8">
+      <c r="C5" s="8"/>
+      <c r="E5" s="9">
         <v>45716</v>
       </c>
-      <c r="F5" s="24"/>
+      <c r="F5" s="25"/>
     </row>
     <row r="6" spans="1:16">
-      <c r="A6" s="5"/>
-      <c r="B6" s="10" t="s">
+      <c r="A6" s="6"/>
+      <c r="B6" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="9"/>
-      <c r="D6" s="22"/>
-      <c r="E6" s="8">
+      <c r="C6" s="10"/>
+      <c r="D6" s="23"/>
+      <c r="E6" s="9">
         <v>45716</v>
       </c>
-      <c r="F6" s="24"/>
+      <c r="F6" s="25"/>
     </row>
     <row r="7" spans="1:16">
-      <c r="A7" s="5">
+      <c r="A7" s="6">
         <v>4</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="11"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8">
+      <c r="C7" s="12"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9">
         <v>45723</v>
       </c>
-      <c r="F7" s="8"/>
+      <c r="F7" s="9"/>
     </row>
     <row r="8" spans="1:16">
-      <c r="A8" s="5">
+      <c r="A8" s="6">
         <v>5</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="11"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8">
+      <c r="C8" s="12"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9">
         <v>45785</v>
       </c>
-      <c r="F8" s="8"/>
+      <c r="F8" s="9"/>
     </row>
     <row r="9" spans="1:16">
-      <c r="A9" s="5">
+      <c r="A9" s="6">
         <v>6</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="11"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8">
+      <c r="C9" s="12"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9">
         <v>45736</v>
       </c>
-      <c r="F9" s="8"/>
+      <c r="F9" s="9"/>
     </row>
     <row r="10" spans="1:16">
-      <c r="A10" s="5">
+      <c r="A10" s="6">
         <v>7</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="11"/>
-      <c r="D10" s="8"/>
-      <c r="F10" s="8"/>
+      <c r="C10" s="12"/>
+      <c r="D10" s="9"/>
+      <c r="F10" s="9"/>
     </row>
     <row r="11" spans="1:16">
-      <c r="A11" s="5">
+      <c r="A11" s="6">
         <v>8</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="C11" s="11"/>
-      <c r="D11" s="8"/>
-      <c r="F11" s="8"/>
+      <c r="C11" s="12"/>
+      <c r="D11" s="9"/>
+      <c r="F11" s="9"/>
     </row>
     <row r="12" spans="1:16">
-      <c r="A12" s="5"/>
-      <c r="B12" s="21" t="s">
+      <c r="A12" s="6"/>
+      <c r="B12" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="C12" s="11"/>
-      <c r="D12" s="8"/>
+      <c r="C12" s="12"/>
+      <c r="D12" s="9"/>
     </row>
     <row r="13" spans="1:16">
-      <c r="A13" s="5">
+      <c r="A13" s="6">
         <v>9</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="11"/>
-      <c r="D13" s="8"/>
-      <c r="F13" s="8"/>
+      <c r="C13" s="12"/>
+      <c r="D13" s="9"/>
+      <c r="F13" s="9"/>
     </row>
     <row r="14" spans="1:16">
-      <c r="A14" s="25">
+      <c r="A14" s="26">
         <v>10</v>
       </c>
-      <c r="B14" s="18" t="s">
+      <c r="B14" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="19"/>
-      <c r="D14" s="8">
+      <c r="C14" s="20"/>
+      <c r="D14" s="9">
         <v>45660</v>
       </c>
     </row>
     <row r="15" spans="1:16">
-      <c r="A15" s="25">
+      <c r="A15" s="26">
         <v>11</v>
       </c>
-      <c r="B15" s="18" t="s">
+      <c r="B15" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="C15" s="19"/>
-      <c r="D15" s="8">
+      <c r="C15" s="20"/>
+      <c r="D15" s="9">
         <v>45667</v>
       </c>
     </row>
     <row r="16" spans="1:16">
-      <c r="A16" s="25">
+      <c r="A16" s="26">
         <v>12</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="C16" s="19"/>
-      <c r="D16" s="8">
+      <c r="C16" s="20"/>
+      <c r="D16" s="9">
         <v>45674</v>
       </c>
-      <c r="F16" s="8"/>
+      <c r="F16" s="9"/>
     </row>
     <row r="17" spans="1:7">
-      <c r="A17" s="25">
+      <c r="A17" s="26">
         <v>13</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="C17" s="11"/>
-      <c r="D17" s="8">
+      <c r="C17" s="12"/>
+      <c r="D17" s="9">
         <v>45681</v>
       </c>
-      <c r="F17" s="8"/>
+      <c r="F17" s="9"/>
     </row>
     <row r="18" spans="1:7">
-      <c r="A18" s="5">
+      <c r="A18" s="6">
         <v>14</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="B18" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="C18" s="11"/>
-      <c r="D18" s="8">
+      <c r="C18" s="12"/>
+      <c r="D18" s="9">
         <v>45730</v>
       </c>
-      <c r="F18" s="8"/>
+      <c r="F18" s="9"/>
     </row>
     <row r="21" ht="17.4" spans="1:7">
       <c r="A21" s="1" t="s">
@@ -2919,123 +2925,123 @@
       </c>
     </row>
     <row r="22" spans="1:7">
-      <c r="A22" s="4" t="s">
+      <c r="A22" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="5" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="23" spans="1:7">
-      <c r="A23" s="5">
+      <c r="A23" s="6">
         <v>1</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C23" s="5" t="s">
+      <c r="C23" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="D23" s="8"/>
-      <c r="E23" s="8">
+      <c r="D23" s="9"/>
+      <c r="E23" s="9">
         <v>45681</v>
       </c>
-      <c r="F23" s="8">
+      <c r="F23" s="9">
         <v>45723</v>
       </c>
-      <c r="G23" s="8">
+      <c r="G23" s="9">
         <v>45765</v>
       </c>
     </row>
     <row r="24" spans="1:7">
-      <c r="A24" s="5">
+      <c r="A24" s="6">
         <v>3</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="B24" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C24" s="7" t="s">
+      <c r="C24" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="D24" s="8">
+      <c r="D24" s="9">
         <v>45660</v>
       </c>
-      <c r="E24" s="8">
+      <c r="E24" s="9">
         <v>45701</v>
       </c>
-      <c r="F24" s="8">
+      <c r="F24" s="9">
         <v>45730</v>
       </c>
     </row>
     <row r="25" spans="1:7">
-      <c r="A25" s="5">
+      <c r="A25" s="6">
         <v>4</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C25" s="9"/>
-      <c r="D25" s="8">
+      <c r="C25" s="10"/>
+      <c r="D25" s="9">
         <v>45660</v>
       </c>
-      <c r="E25" s="8">
+      <c r="E25" s="9">
         <v>45701</v>
       </c>
-      <c r="F25" s="8">
+      <c r="F25" s="9">
         <v>45730</v>
       </c>
     </row>
     <row r="26" spans="1:7">
-      <c r="A26" s="5">
+      <c r="A26" s="6">
         <v>2</v>
       </c>
-      <c r="B26" s="6" t="s">
+      <c r="B26" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="C26" s="5" t="s">
+      <c r="C26" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="D26" s="8">
+      <c r="D26" s="9">
         <v>45667</v>
       </c>
-      <c r="E26" s="8">
+      <c r="E26" s="9">
         <v>45709</v>
       </c>
-      <c r="F26" s="8">
+      <c r="F26" s="9">
         <v>45736</v>
       </c>
     </row>
     <row r="27" spans="1:7">
-      <c r="A27" s="5">
+      <c r="A27" s="6">
         <v>5</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C27" s="5" t="s">
+      <c r="C27" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="D27" s="8">
+      <c r="D27" s="9">
         <v>45674</v>
       </c>
-      <c r="E27" s="8">
+      <c r="E27" s="9">
         <v>45716</v>
       </c>
-      <c r="F27" s="8">
+      <c r="F27" s="9">
         <v>45759</v>
       </c>
     </row>
     <row r="28" spans="1:7">
-      <c r="B28" s="10" t="s">
+      <c r="B28" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="C28" s="11" t="s">
+      <c r="C28" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="F28" s="8">
+      <c r="F28" s="9">
         <v>45743</v>
       </c>
     </row>
@@ -3076,437 +3082,444 @@
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="3"/>
+      <c r="D1" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
       <c r="H1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="5">
+      <c r="A3" s="6">
         <v>1</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="9">
         <v>45660</v>
       </c>
-      <c r="E3" s="8">
+      <c r="E3" s="9">
         <v>45701</v>
       </c>
-      <c r="F3" s="8">
+      <c r="F3" s="9">
         <v>45730</v>
       </c>
-      <c r="G3" s="8">
+      <c r="G3" s="9">
         <v>45891</v>
       </c>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="5">
+      <c r="A4" s="6">
         <v>2</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C4" s="9"/>
-      <c r="D4" s="8">
+      <c r="C4" s="10"/>
+      <c r="D4" s="9">
         <v>45660</v>
       </c>
-      <c r="E4" s="8">
+      <c r="E4" s="9">
         <v>45701</v>
       </c>
-      <c r="F4" s="8">
+      <c r="F4" s="9">
         <v>45730</v>
       </c>
-      <c r="G4" s="8">
+      <c r="G4" s="9">
         <v>45891</v>
       </c>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="5">
+      <c r="A5" s="6">
         <v>3</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="D5" s="8">
+      <c r="D5" s="9">
         <v>45667</v>
       </c>
-      <c r="E5" s="8">
+      <c r="E5" s="9">
         <v>45709</v>
       </c>
-      <c r="F5" s="8">
+      <c r="F5" s="9">
         <v>45736</v>
       </c>
-      <c r="G5" s="8">
+      <c r="G5" s="9">
         <v>45912</v>
       </c>
     </row>
     <row r="6" spans="1:8">
-      <c r="A6" s="5">
+      <c r="A6" s="6">
         <v>4</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="9">
         <v>45674</v>
       </c>
-      <c r="E6" s="8">
+      <c r="E6" s="9">
         <v>45716</v>
       </c>
-      <c r="F6" s="8">
+      <c r="F6" s="9">
         <v>45759</v>
       </c>
-      <c r="G6" s="8">
+      <c r="G6" s="9">
         <v>45897</v>
       </c>
     </row>
     <row r="7" spans="1:8">
-      <c r="A7" s="5">
+      <c r="A7" s="6">
         <v>5</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="D7" s="8">
+      <c r="D7" s="9">
         <v>45681</v>
       </c>
-      <c r="E7" s="8">
+      <c r="E7" s="9">
         <v>45723</v>
       </c>
-      <c r="F7" s="8">
+      <c r="F7" s="9">
         <v>45765</v>
       </c>
-      <c r="G7" s="8">
+      <c r="G7" s="9">
         <v>45905</v>
       </c>
     </row>
     <row r="8" spans="1:8">
-      <c r="A8" s="5">
+      <c r="A8" s="6">
         <v>6</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="11"/>
-      <c r="D8" s="8"/>
-      <c r="F8" s="8">
+      <c r="C8" s="12"/>
+      <c r="D8" s="9"/>
+      <c r="F8" s="9">
         <v>45785</v>
       </c>
       <c r="G8" t="s">
-        <v>63</v>
-      </c>
-      <c r="H8" s="8">
+        <v>64</v>
+      </c>
+      <c r="H8" s="9">
         <v>46101</v>
       </c>
     </row>
     <row r="9" spans="1:8">
-      <c r="A9" s="5">
+      <c r="A9" s="6">
         <v>7</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="C9" s="11"/>
-      <c r="D9" s="8"/>
-      <c r="F9" s="8">
+      <c r="C9" s="12"/>
+      <c r="D9" s="9"/>
+      <c r="F9" s="9">
         <v>45793</v>
       </c>
-      <c r="G9" s="8">
+      <c r="G9" s="9">
         <v>45954</v>
       </c>
     </row>
     <row r="10" spans="1:8">
-      <c r="A10" s="5">
+      <c r="A10" s="6">
         <v>8</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="11"/>
-      <c r="D10" s="8"/>
-      <c r="F10" s="8">
+      <c r="C10" s="12"/>
+      <c r="D10" s="9"/>
+      <c r="F10" s="9">
         <v>45800</v>
       </c>
-      <c r="G10" s="8">
+      <c r="G10" s="9">
         <v>45961</v>
       </c>
     </row>
     <row r="11" ht="15.6" spans="1:8">
-      <c r="A11" s="7">
+      <c r="A11" s="8">
         <v>9</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="B11" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="C11" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="D11" s="14" t="s">
+      <c r="D11" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="F11" s="8">
+      <c r="F11" s="9">
         <v>45806</v>
       </c>
-      <c r="H11" s="8">
+      <c r="H11" s="9">
         <v>46084</v>
       </c>
     </row>
     <row r="12" ht="15.6" spans="1:8">
-      <c r="A12" s="15"/>
-      <c r="B12" s="16"/>
-      <c r="C12" s="13" t="s">
+      <c r="A12" s="16"/>
+      <c r="B12" s="17"/>
+      <c r="C12" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="D12" s="14" t="s">
+      <c r="D12" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="F12" s="8">
+      <c r="F12" s="9">
         <v>45743</v>
       </c>
     </row>
     <row r="13" ht="15.6" spans="1:8">
-      <c r="A13" s="9"/>
-      <c r="B13" s="17"/>
-      <c r="C13" s="13" t="s">
+      <c r="A13" s="10"/>
+      <c r="B13" s="18"/>
+      <c r="C13" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="D13" s="14" t="s">
+      <c r="D13" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8">
+      <c r="F13" s="9"/>
+      <c r="G13" s="9">
         <v>45959</v>
       </c>
     </row>
     <row r="14" spans="1:8">
-      <c r="A14" s="5">
+      <c r="A14" s="6">
         <v>10</v>
       </c>
-      <c r="B14" s="18" t="s">
+      <c r="B14" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="19"/>
-      <c r="D14" s="8"/>
-      <c r="F14" s="8">
+      <c r="C14" s="20"/>
+      <c r="D14" s="9"/>
+      <c r="F14" s="9">
         <v>45814</v>
       </c>
-      <c r="G14" s="8">
+      <c r="G14" s="9">
         <v>45975</v>
       </c>
     </row>
     <row r="15" spans="1:8">
-      <c r="A15" s="5">
+      <c r="A15" s="6">
         <v>11</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="B15" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="C15" s="11"/>
-      <c r="D15" s="8"/>
-      <c r="F15" s="20">
+      <c r="C15" s="12"/>
+      <c r="D15" s="9"/>
+      <c r="F15" s="21">
         <v>45821</v>
       </c>
-      <c r="G15" s="8">
+      <c r="G15" s="9">
         <v>45982</v>
       </c>
     </row>
     <row r="16" spans="1:8">
-      <c r="A16" s="5">
+      <c r="A16" s="6">
         <v>12</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="C16" s="11"/>
-      <c r="D16" s="8"/>
-      <c r="F16" s="8">
+      <c r="C16" s="12"/>
+      <c r="D16" s="9"/>
+      <c r="F16" s="9">
         <v>45828</v>
       </c>
-      <c r="G16" s="8">
+      <c r="G16" s="9">
         <v>45989</v>
       </c>
     </row>
-    <row r="17" spans="1:7">
-      <c r="A17" s="5">
+    <row r="17" spans="1:8">
+      <c r="A17" s="6">
         <v>13</v>
       </c>
-      <c r="B17" s="21" t="s">
+      <c r="B17" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="C17" s="11"/>
-      <c r="D17" s="8"/>
-      <c r="F17" s="8">
+      <c r="C17" s="12"/>
+      <c r="D17" s="9"/>
+      <c r="F17" s="9">
         <v>45834</v>
       </c>
-      <c r="G17" s="8">
+      <c r="G17" s="9">
         <v>45996</v>
       </c>
     </row>
-    <row r="18" spans="1:7">
-      <c r="A18" s="7">
+    <row r="18" spans="1:8">
+      <c r="A18" s="8">
         <v>14</v>
       </c>
-      <c r="B18" s="11" t="s">
+      <c r="B18" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="C18" s="7"/>
-      <c r="F18" s="8"/>
-      <c r="G18" s="8">
+      <c r="C18" s="8"/>
+      <c r="F18" s="9"/>
+      <c r="H18" s="9">
         <v>45666</v>
       </c>
     </row>
-    <row r="19" spans="1:7">
-      <c r="A19" s="9"/>
-      <c r="B19" s="10" t="s">
+    <row r="19" spans="1:8">
+      <c r="A19" s="10"/>
+      <c r="B19" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C19" s="9"/>
-      <c r="D19" s="22"/>
-      <c r="F19" s="8"/>
-      <c r="G19" s="8">
+      <c r="C19" s="10"/>
+      <c r="D19" s="23"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="9">
         <v>46017</v>
       </c>
     </row>
-    <row r="20" spans="1:7">
-      <c r="A20" s="5">
+    <row r="20" spans="1:8">
+      <c r="A20" s="6">
         <v>15</v>
       </c>
-      <c r="B20" s="10" t="s">
+      <c r="B20" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="C20" s="11"/>
-      <c r="D20" s="8"/>
-      <c r="F20" s="8">
+      <c r="C20" s="12"/>
+      <c r="D20" s="9"/>
+      <c r="F20" s="9">
         <v>45842</v>
       </c>
-      <c r="G20" s="8">
+      <c r="G20" s="9">
         <v>46010</v>
       </c>
     </row>
-    <row r="21" spans="1:7">
-      <c r="A21" s="5">
+    <row r="21" spans="1:8">
+      <c r="A21" s="6">
         <v>16</v>
       </c>
-      <c r="B21" s="10" t="s">
+      <c r="B21" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="C21" s="11"/>
-      <c r="D21" s="8"/>
-      <c r="E21" s="8"/>
-      <c r="F21" s="8">
+      <c r="C21" s="12"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9">
         <v>45849</v>
       </c>
-      <c r="G21" s="8">
+      <c r="H21" s="9">
         <v>46038</v>
       </c>
     </row>
-    <row r="22" spans="1:7">
-      <c r="A22" s="5">
+    <row r="22" spans="1:8">
+      <c r="A22" s="6">
         <v>17</v>
       </c>
-      <c r="B22" s="10" t="s">
+      <c r="B22" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="C22" s="11"/>
-      <c r="D22" s="8"/>
-      <c r="F22" s="8">
+      <c r="C22" s="12"/>
+      <c r="D22" s="9"/>
+      <c r="F22" s="9">
         <v>45856</v>
       </c>
-      <c r="G22" s="8">
+      <c r="H22" s="9">
         <v>46044</v>
       </c>
     </row>
-    <row r="23" spans="1:7">
-      <c r="A23" s="5">
+    <row r="23" spans="1:8">
+      <c r="A23" s="6">
         <v>18</v>
       </c>
-      <c r="B23" s="18" t="s">
+      <c r="B23" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="C23" s="19"/>
-      <c r="D23" s="8"/>
-      <c r="F23" s="8">
+      <c r="C23" s="20"/>
+      <c r="D23" s="9"/>
+      <c r="F23" s="9">
         <v>45863</v>
       </c>
-      <c r="G23" s="8">
+      <c r="H23" s="9">
         <v>46087</v>
       </c>
     </row>
-    <row r="24" spans="1:7">
-      <c r="A24" s="5">
+    <row r="24" spans="1:8">
+      <c r="A24" s="6">
         <v>19</v>
       </c>
-      <c r="B24" s="10" t="s">
+      <c r="B24" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="C24" s="19"/>
-      <c r="D24" s="8"/>
-      <c r="F24" s="8">
+      <c r="C24" s="20"/>
+      <c r="D24" s="9"/>
+      <c r="F24" s="9">
         <v>45870</v>
       </c>
-      <c r="G24" s="8">
+      <c r="H24" s="9">
         <v>46094</v>
       </c>
     </row>
-    <row r="25" spans="1:7">
-      <c r="A25" s="5">
+    <row r="25" spans="1:8">
+      <c r="A25" s="6">
         <v>20</v>
       </c>
-      <c r="B25" s="10" t="s">
+      <c r="B25" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="C25" s="11"/>
-      <c r="D25" s="8"/>
-      <c r="F25" s="8">
+      <c r="C25" s="12"/>
+      <c r="D25" s="9"/>
+      <c r="F25" s="9">
         <v>45877</v>
       </c>
-      <c r="G25" s="8">
+      <c r="H25" s="9">
         <v>46108</v>
       </c>
     </row>
-    <row r="26" spans="1:7">
-      <c r="A26" s="5">
+    <row r="26" spans="1:8">
+      <c r="A26" s="6">
         <v>21</v>
       </c>
-      <c r="B26" s="10" t="s">
+      <c r="B26" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="C26" s="11"/>
-      <c r="D26" s="8"/>
-      <c r="F26" s="8">
+      <c r="C26" s="12"/>
+      <c r="D26" s="9"/>
+      <c r="F26" s="9">
         <v>45884</v>
       </c>
-      <c r="G26" s="8">
+      <c r="H26" s="9">
         <v>46058</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="A1:C1"/>
+    <mergeCell ref="D1:G1"/>
     <mergeCell ref="A11:A13"/>
     <mergeCell ref="A18:A19"/>
     <mergeCell ref="B11:B13"/>

</xml_diff>